<commit_message>
feat: bind 24 Kstat slots to quota items and enable web UI pilot and batch execution
</commit_message>
<xml_diff>
--- a/data/quotas/quota_onnuri_2026_풍납시장_업종별24개_조사쿼터_1792039611646.xlsx
+++ b/data/quotas/quota_onnuri_2026_풍납시장_업종별24개_조사쿼터_1792039611646.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <workbookPr codeName="ThisWorkbook"/>
   <sheets>
-    <sheet name="조사쿼터_사업자목록" sheetId="1" r:id="rId1"/>
+    <sheet name="풍납시장_24개_Kstat매핑" sheetId="1" r:id="rId1"/>
   </sheets>
 </workbook>
 </file>
@@ -397,58 +397,50 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:L25"/>
-  <cols>
-    <col min="1" max="1" width="10.83203125" customWidth="1"/>
-    <col min="2" max="2" width="11.83203125" customWidth="1"/>
-    <col min="3" max="3" width="31.83203125" customWidth="1"/>
-    <col min="4" max="4" width="19.234375" customWidth="1"/>
-    <col min="5" max="5" width="12.6328125" customWidth="1"/>
-    <col min="6" max="6" width="17.83203125" customWidth="1"/>
-    <col min="7" max="7" width="13.83203125" customWidth="1"/>
-    <col min="8" max="8" width="55.83203125" customWidth="1"/>
-    <col min="9" max="9" width="34.83203125" customWidth="1"/>
-    <col min="10" max="10" width="12.6328125" customWidth="1"/>
-    <col min="11" max="11" width="14.83203125" customWidth="1"/>
-    <col min="12" max="12" width="17.03515625" customWidth="1"/>
-  </cols>
+  <dimension ref="A1:N25"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
-        <v>No</v>
+        <v>순번</v>
       </c>
       <c r="B1" t="str">
+        <v>Kstat슬롯</v>
+      </c>
+      <c r="C1" t="str">
+        <v>Kstat설문URL</v>
+      </c>
+      <c r="D1" t="str">
         <v>시장명</v>
       </c>
-      <c r="C1" t="str">
-        <v>상호(가맹점명)</v>
-      </c>
-      <c r="D1" t="str">
-        <v>사업자등록번호</v>
-      </c>
       <c r="E1" t="str">
+        <v>상호</v>
+      </c>
+      <c r="F1" t="str">
+        <v>사업자번호</v>
+      </c>
+      <c r="G1" t="str">
         <v>대표자명</v>
       </c>
-      <c r="F1" t="str">
+      <c r="H1" t="str">
         <v>연락처</v>
       </c>
-      <c r="G1" t="str">
-        <v>개업연월</v>
-      </c>
-      <c r="H1" t="str">
-        <v>취급품목(업종)</v>
-      </c>
       <c r="I1" t="str">
-        <v>주소</v>
+        <v>개업일</v>
       </c>
       <c r="J1" t="str">
+        <v>업종/품목</v>
+      </c>
+      <c r="K1" t="str">
+        <v>사업장주소</v>
+      </c>
+      <c r="L1" t="str">
         <v>가맹상태</v>
       </c>
-      <c r="K1" t="str">
-        <v>온누리지류</v>
-      </c>
-      <c r="L1" t="str">
-        <v>온누리디지털</v>
+      <c r="M1" t="str">
+        <v>지류</v>
+      </c>
+      <c r="N1" t="str">
+        <v>디지털</v>
       </c>
     </row>
     <row r="2" xml:space="preserve">
@@ -456,37 +448,43 @@
         <v>1</v>
       </c>
       <c r="B2" t="str">
-        <v>풍납시장</v>
+        <v>슬롯 #2 (4)추가</v>
       </c>
       <c r="C2" t="str">
+        <v>https://kstat.surveys.kr/2026/P26042401B/index.asp?KID=EZQPGx4L8&amp;type=tapi&amp;prid=2026070802&amp;mnid=900001346&amp;srt=1</v>
+      </c>
+      <c r="D2" t="str">
+        <v>풍납시장</v>
+      </c>
+      <c r="E2" t="str">
         <v>더덕상회</v>
       </c>
-      <c r="D2" t="str">
+      <c r="F2" t="str">
         <v>626-22-02194</v>
       </c>
-      <c r="E2" t="str">
+      <c r="G2" t="str">
         <v>이은지</v>
       </c>
-      <c r="F2" t="str">
+      <c r="H2" t="str">
         <v>02-484-4953</v>
       </c>
-      <c r="G2" t="str">
+      <c r="I2" t="str">
         <v>2025-12-24</v>
       </c>
-      <c r="H2" t="str">
+      <c r="J2" t="str">
         <v>농산물 (곡물)</v>
       </c>
-      <c r="I2" t="str" xml:space="preserve">
-        <v xml:space="preserve">서울특별시 송파구
-주소정보 갱신</v>
-      </c>
-      <c r="J2" t="str">
-        <v>정상가맹</v>
-      </c>
-      <c r="K2" t="str">
-        <v>Y</v>
+      <c r="K2" t="str" xml:space="preserve">
+        <v xml:space="preserve">서울특별시 송파구
+주소정보 갱신</v>
       </c>
       <c r="L2" t="str">
+        <v>정상가맹</v>
+      </c>
+      <c r="M2" t="str">
+        <v>Y</v>
+      </c>
+      <c r="N2" t="str">
         <v>Y</v>
       </c>
     </row>
@@ -495,37 +493,43 @@
         <v>2</v>
       </c>
       <c r="B3" t="str">
-        <v>풍납시장</v>
+        <v>슬롯 #3 (5)추가</v>
       </c>
       <c r="C3" t="str">
+        <v>https://kstat.surveys.kr/2026/P26042401B/index.asp?KID=VCnUfCY6K&amp;type=tapi&amp;prid=2026070802&amp;mnid=900001346&amp;srt=1</v>
+      </c>
+      <c r="D3" t="str">
+        <v>풍납시장</v>
+      </c>
+      <c r="E3" t="str">
         <v>정주상회</v>
       </c>
-      <c r="D3" t="str">
+      <c r="F3" t="str">
         <v>219-99-00710</v>
       </c>
-      <c r="E3" t="str">
-        <v/>
-      </c>
-      <c r="F3" t="str">
+      <c r="G3" t="str">
+        <v>-</v>
+      </c>
+      <c r="H3" t="str">
         <v>02-414-8784</v>
       </c>
-      <c r="G3" t="str">
+      <c r="I3" t="str">
         <v>2013-05-28</v>
       </c>
-      <c r="H3" t="str">
+      <c r="J3" t="str">
         <v>농산물 (통신ㆍ방송장비 및 부품 도매업 외 1개)</v>
       </c>
-      <c r="I3" t="str" xml:space="preserve">
-        <v xml:space="preserve">서울특별시 송파구
-주소정보 갱신</v>
-      </c>
-      <c r="J3" t="str">
-        <v>정상가맹</v>
-      </c>
-      <c r="K3" t="str">
-        <v>Y</v>
+      <c r="K3" t="str" xml:space="preserve">
+        <v xml:space="preserve">서울특별시 송파구
+주소정보 갱신</v>
       </c>
       <c r="L3" t="str">
+        <v>정상가맹</v>
+      </c>
+      <c r="M3" t="str">
+        <v>Y</v>
+      </c>
+      <c r="N3" t="str">
         <v>Y</v>
       </c>
     </row>
@@ -534,37 +538,43 @@
         <v>3</v>
       </c>
       <c r="B4" t="str">
-        <v>풍납시장</v>
+        <v>슬롯 #4 (6)추가</v>
       </c>
       <c r="C4" t="str">
+        <v>https://kstat.surveys.kr/2026/P26042401B/index.asp?KID=05anItSeU&amp;type=tapi&amp;prid=2026070802&amp;mnid=900001346&amp;srt=1</v>
+      </c>
+      <c r="D4" t="str">
+        <v>풍납시장</v>
+      </c>
+      <c r="E4" t="str">
         <v>세일축산</v>
       </c>
-      <c r="D4" t="str">
+      <c r="F4" t="str">
         <v>230-90-07847</v>
       </c>
-      <c r="E4" t="str">
-        <v/>
-      </c>
-      <c r="F4" t="str">
+      <c r="G4" t="str">
+        <v>-</v>
+      </c>
+      <c r="H4" t="str">
         <v>010-012-0001</v>
       </c>
-      <c r="G4" t="str">
+      <c r="I4" t="str">
         <v>2014-09-23</v>
       </c>
-      <c r="H4" t="str">
+      <c r="J4" t="str">
         <v>축산물 (육류 소매업)</v>
       </c>
-      <c r="I4" t="str" xml:space="preserve">
-        <v xml:space="preserve">서울특별시 송파구
-주소정보 갱신</v>
-      </c>
-      <c r="J4" t="str">
-        <v>정상가맹</v>
-      </c>
-      <c r="K4" t="str">
-        <v>Y</v>
+      <c r="K4" t="str" xml:space="preserve">
+        <v xml:space="preserve">서울특별시 송파구
+주소정보 갱신</v>
       </c>
       <c r="L4" t="str">
+        <v>정상가맹</v>
+      </c>
+      <c r="M4" t="str">
+        <v>Y</v>
+      </c>
+      <c r="N4" t="str">
         <v>Y</v>
       </c>
     </row>
@@ -573,36 +583,42 @@
         <v>4</v>
       </c>
       <c r="B5" t="str">
-        <v>풍납시장</v>
+        <v>슬롯 #5 (1)추가</v>
       </c>
       <c r="C5" t="str">
+        <v>https://kstat.surveys.kr/2026/P26042401B/index.asp?KID=0E6G9JX98&amp;type=tapi&amp;prid=2026070802&amp;mnid=900001346&amp;srt=1</v>
+      </c>
+      <c r="D5" t="str">
+        <v>풍납시장</v>
+      </c>
+      <c r="E5" t="str">
         <v>한우마을</v>
       </c>
-      <c r="D5" t="str">
+      <c r="F5" t="str">
         <v>501-92-55721</v>
       </c>
-      <c r="E5" t="str">
-        <v/>
-      </c>
-      <c r="F5" t="str">
+      <c r="G5" t="str">
+        <v>-</v>
+      </c>
+      <c r="H5" t="str">
         <v>02-482-6192</v>
       </c>
-      <c r="G5" t="str">
+      <c r="I5" t="str">
         <v>2017-03-21</v>
       </c>
-      <c r="H5" t="str">
+      <c r="J5" t="str">
         <v>축산물 (육류 도매업 외 1개)</v>
       </c>
-      <c r="I5" t="str">
+      <c r="K5" t="str">
         <v>서울특별시 송파구</v>
       </c>
-      <c r="J5" t="str">
-        <v>정상가맹</v>
-      </c>
-      <c r="K5" t="str">
-        <v>Y</v>
-      </c>
       <c r="L5" t="str">
+        <v>정상가맹</v>
+      </c>
+      <c r="M5" t="str">
+        <v>Y</v>
+      </c>
+      <c r="N5" t="str">
         <v>Y</v>
       </c>
     </row>
@@ -611,36 +627,42 @@
         <v>5</v>
       </c>
       <c r="B6" t="str">
-        <v>풍납시장</v>
+        <v>슬롯 #6 (2)추가</v>
       </c>
       <c r="C6" t="str">
+        <v>https://kstat.surveys.kr/2026/P26042401B/index.asp?KID=OseLErRyW&amp;type=tapi&amp;prid=2026070802&amp;mnid=900001346&amp;srt=1</v>
+      </c>
+      <c r="D6" t="str">
+        <v>풍납시장</v>
+      </c>
+      <c r="E6" t="str">
         <v>칠칠수산</v>
       </c>
-      <c r="D6" t="str">
+      <c r="F6" t="str">
         <v>555-95-01465</v>
       </c>
-      <c r="E6" t="str">
+      <c r="G6" t="str">
         <v>오지은</v>
       </c>
-      <c r="F6" t="str">
+      <c r="H6" t="str">
         <v>0507-1332-3533</v>
       </c>
-      <c r="G6" t="str">
+      <c r="I6" t="str">
         <v>2020-10-22</v>
       </c>
-      <c r="H6" t="str">
+      <c r="J6" t="str">
         <v>수산물 (신선)</v>
       </c>
-      <c r="I6" t="str">
+      <c r="K6" t="str">
         <v>서울특별시 송파구</v>
       </c>
-      <c r="J6" t="str">
-        <v>정상가맹</v>
-      </c>
-      <c r="K6" t="str">
-        <v>Y</v>
-      </c>
       <c r="L6" t="str">
+        <v>정상가맹</v>
+      </c>
+      <c r="M6" t="str">
+        <v>Y</v>
+      </c>
+      <c r="N6" t="str">
         <v>N</v>
       </c>
     </row>
@@ -649,37 +671,43 @@
         <v>6</v>
       </c>
       <c r="B7" t="str">
-        <v>풍납시장</v>
+        <v>슬롯 #7 (7)추가</v>
       </c>
       <c r="C7" t="str">
+        <v>https://kstat.surveys.kr/2026/P26042401B/index.asp?KID=9VS1l8O1Y&amp;type=tapi&amp;prid=2026070802&amp;mnid=900001346&amp;srt=1</v>
+      </c>
+      <c r="D7" t="str">
+        <v>풍납시장</v>
+      </c>
+      <c r="E7" t="str">
         <v>물고기</v>
       </c>
-      <c r="D7" t="str">
+      <c r="F7" t="str">
         <v>183-95-01483</v>
       </c>
-      <c r="E7" t="str">
-        <v/>
-      </c>
-      <c r="F7" t="str">
+      <c r="G7" t="str">
+        <v>-</v>
+      </c>
+      <c r="H7" t="str">
         <v>0507-1332-3533</v>
       </c>
-      <c r="G7" t="str">
+      <c r="I7" t="str">
         <v>2022-04-22</v>
       </c>
-      <c r="H7" t="str">
+      <c r="J7" t="str">
         <v>수산물 (음ㆍ식료품 및 담배 도매업 외 1개)</v>
       </c>
-      <c r="I7" t="str" xml:space="preserve">
-        <v xml:space="preserve">서울특별시 송파구
-주소정보 갱신</v>
-      </c>
-      <c r="J7" t="str">
-        <v>정상가맹</v>
-      </c>
-      <c r="K7" t="str">
-        <v>Y</v>
+      <c r="K7" t="str" xml:space="preserve">
+        <v xml:space="preserve">서울특별시 송파구
+주소정보 갱신</v>
       </c>
       <c r="L7" t="str">
+        <v>정상가맹</v>
+      </c>
+      <c r="M7" t="str">
+        <v>Y</v>
+      </c>
+      <c r="N7" t="str">
         <v>Y</v>
       </c>
     </row>
@@ -688,37 +716,43 @@
         <v>7</v>
       </c>
       <c r="B8" t="str">
-        <v>풍납시장</v>
+        <v>슬롯 #8 (3)추가</v>
       </c>
       <c r="C8" t="str">
+        <v>https://kstat.surveys.kr/2026/P26042401B/index.asp?KID=yJOWyMMVe&amp;type=tapi&amp;prid=2026070802&amp;mnid=900001346&amp;srt=1</v>
+      </c>
+      <c r="D8" t="str">
+        <v>풍납시장</v>
+      </c>
+      <c r="E8" t="str">
         <v>뻥튀기가 맛있는 집</v>
       </c>
-      <c r="D8" t="str">
+      <c r="F8" t="str">
         <v>381-65-00776</v>
       </c>
-      <c r="E8" t="str">
-        <v/>
-      </c>
-      <c r="F8" t="str">
+      <c r="G8" t="str">
+        <v>-</v>
+      </c>
+      <c r="H8" t="str">
         <v>02-403-8822</v>
       </c>
-      <c r="G8" t="str">
+      <c r="I8" t="str">
         <v>2025-07-16</v>
       </c>
-      <c r="H8" t="str">
+      <c r="J8" t="str">
         <v>가공식품 (그 외 기타 분류 안된 상품 전문 소매업)</v>
       </c>
-      <c r="I8" t="str" xml:space="preserve">
-        <v xml:space="preserve">서울특별시 송파구
-주소정보 갱신</v>
-      </c>
-      <c r="J8" t="str">
-        <v>정상가맹</v>
-      </c>
-      <c r="K8" t="str">
-        <v>Y</v>
+      <c r="K8" t="str" xml:space="preserve">
+        <v xml:space="preserve">서울특별시 송파구
+주소정보 갱신</v>
       </c>
       <c r="L8" t="str">
+        <v>정상가맹</v>
+      </c>
+      <c r="M8" t="str">
+        <v>Y</v>
+      </c>
+      <c r="N8" t="str">
         <v>Y</v>
       </c>
     </row>
@@ -727,37 +761,43 @@
         <v>8</v>
       </c>
       <c r="B9" t="str">
-        <v>풍납시장</v>
+        <v>슬롯 #9 (8)추가</v>
       </c>
       <c r="C9" t="str">
+        <v>https://kstat.surveys.kr/2026/P26042401B/index.asp?KID=l72YcIVMm&amp;type=tapi&amp;prid=2026070802&amp;mnid=900001346&amp;srt=1</v>
+      </c>
+      <c r="D9" t="str">
+        <v>풍납시장</v>
+      </c>
+      <c r="E9" t="str">
         <v>양지기름</v>
       </c>
-      <c r="D9" t="str">
+      <c r="F9" t="str">
         <v>219-01-40388</v>
       </c>
-      <c r="E9" t="str">
+      <c r="G9" t="str">
         <v>조용수</v>
       </c>
-      <c r="F9" t="str">
+      <c r="H9" t="str">
         <v>02-2147-4540</v>
       </c>
-      <c r="G9" t="str">
+      <c r="I9" t="str">
         <v>2011-05-12</v>
       </c>
-      <c r="H9" t="str">
+      <c r="J9" t="str">
         <v>가공식품 (동ㆍ식물성 유지 및 낙농제품 제조업 외 1개)</v>
       </c>
-      <c r="I9" t="str" xml:space="preserve">
-        <v xml:space="preserve">서울특별시 송파구
-주소정보 갱신</v>
-      </c>
-      <c r="J9" t="str">
-        <v>정상가맹</v>
-      </c>
-      <c r="K9" t="str">
-        <v>Y</v>
+      <c r="K9" t="str" xml:space="preserve">
+        <v xml:space="preserve">서울특별시 송파구
+주소정보 갱신</v>
       </c>
       <c r="L9" t="str">
+        <v>정상가맹</v>
+      </c>
+      <c r="M9" t="str">
+        <v>Y</v>
+      </c>
+      <c r="N9" t="str">
         <v>Y</v>
       </c>
     </row>
@@ -766,37 +806,43 @@
         <v>9</v>
       </c>
       <c r="B10" t="str">
-        <v>풍납시장</v>
+        <v>슬롯 #10 (9)추가</v>
       </c>
       <c r="C10" t="str">
+        <v>https://kstat.surveys.kr/2026/P26042401B/index.asp?KID=BtQ09ixb5&amp;type=tapi&amp;prid=2026070802&amp;mnid=900001346&amp;srt=1</v>
+      </c>
+      <c r="D10" t="str">
+        <v>풍납시장</v>
+      </c>
+      <c r="E10" t="str">
         <v>백군떡방</v>
       </c>
-      <c r="D10" t="str">
+      <c r="F10" t="str">
         <v>230-01-02611</v>
       </c>
-      <c r="E10" t="str">
-        <v/>
-      </c>
-      <c r="F10" t="str">
+      <c r="G10" t="str">
+        <v>-</v>
+      </c>
+      <c r="H10" t="str">
         <v>02-2202-1002</v>
       </c>
-      <c r="G10" t="str">
+      <c r="I10" t="str">
         <v>2022-06-27</v>
       </c>
-      <c r="H10" t="str">
+      <c r="J10" t="str">
         <v>가공식품 (도시락 및 식사용 조리식품 제조업)</v>
       </c>
-      <c r="I10" t="str" xml:space="preserve">
-        <v xml:space="preserve">서울특별시 송파구
-주소정보 갱신</v>
-      </c>
-      <c r="J10" t="str">
-        <v>정상가맹</v>
-      </c>
-      <c r="K10" t="str">
-        <v>Y</v>
+      <c r="K10" t="str" xml:space="preserve">
+        <v xml:space="preserve">서울특별시 송파구
+주소정보 갱신</v>
       </c>
       <c r="L10" t="str">
+        <v>정상가맹</v>
+      </c>
+      <c r="M10" t="str">
+        <v>Y</v>
+      </c>
+      <c r="N10" t="str">
         <v>Y</v>
       </c>
     </row>
@@ -805,37 +851,43 @@
         <v>10</v>
       </c>
       <c r="B11" t="str">
-        <v>풍납시장</v>
+        <v>슬롯 #11 (10)추가</v>
       </c>
       <c r="C11" t="str">
+        <v>https://kstat.surveys.kr/2026/P26042401B/index.asp?KID=Nn9f36TCG&amp;type=tapi&amp;prid=2026070802&amp;mnid=900001346&amp;srt=1</v>
+      </c>
+      <c r="D11" t="str">
+        <v>풍납시장</v>
+      </c>
+      <c r="E11" t="str">
         <v>오뜨레</v>
       </c>
-      <c r="D11" t="str">
+      <c r="F11" t="str">
         <v>104-07-37720</v>
       </c>
-      <c r="E11" t="str">
-        <v/>
-      </c>
-      <c r="F11" t="str">
+      <c r="G11" t="str">
+        <v>-</v>
+      </c>
+      <c r="H11" t="str">
         <v>02-471-0589</v>
       </c>
-      <c r="G11" t="str">
+      <c r="I11" t="str">
         <v>2017-03-21</v>
       </c>
-      <c r="H11" t="str">
+      <c r="J11" t="str">
         <v>의류신발 (여자용 겉옷 소매업 외 1개)</v>
       </c>
-      <c r="I11" t="str" xml:space="preserve">
-        <v xml:space="preserve">서울특별시 송파구
-주소정보 갱신</v>
-      </c>
-      <c r="J11" t="str">
-        <v>정상가맹</v>
-      </c>
-      <c r="K11" t="str">
-        <v>Y</v>
+      <c r="K11" t="str" xml:space="preserve">
+        <v xml:space="preserve">서울특별시 송파구
+주소정보 갱신</v>
       </c>
       <c r="L11" t="str">
+        <v>정상가맹</v>
+      </c>
+      <c r="M11" t="str">
+        <v>Y</v>
+      </c>
+      <c r="N11" t="str">
         <v>Y</v>
       </c>
     </row>
@@ -844,36 +896,42 @@
         <v>11</v>
       </c>
       <c r="B12" t="str">
-        <v>풍납시장</v>
+        <v>슬롯 #12 (11)추가</v>
       </c>
       <c r="C12" t="str">
+        <v>https://kstat.surveys.kr/2026/P26042401B/index.asp?KID=GmWo8WUiG&amp;type=tapi&amp;prid=2026070802&amp;mnid=900001346&amp;srt=1</v>
+      </c>
+      <c r="D12" t="str">
+        <v>풍납시장</v>
+      </c>
+      <c r="E12" t="str">
         <v>올스타</v>
       </c>
-      <c r="D12" t="str">
+      <c r="F12" t="str">
         <v>645-05-03576</v>
       </c>
-      <c r="E12" t="str">
+      <c r="G12" t="str">
         <v>박동원</v>
       </c>
-      <c r="F12" t="str">
+      <c r="H12" t="str">
         <v>02-430-4240</v>
       </c>
-      <c r="G12" t="str">
+      <c r="I12" t="str">
         <v>2025-09-11</v>
       </c>
-      <c r="H12" t="str">
+      <c r="J12" t="str">
         <v>의류신발 (의류/패션잡화/신발 소매)</v>
       </c>
-      <c r="I12" t="str">
+      <c r="K12" t="str">
         <v>서울특별시 송파구 풍납동 1층</v>
       </c>
-      <c r="J12" t="str">
-        <v>정상가맹</v>
-      </c>
-      <c r="K12" t="str">
-        <v>Y</v>
-      </c>
       <c r="L12" t="str">
+        <v>정상가맹</v>
+      </c>
+      <c r="M12" t="str">
+        <v>Y</v>
+      </c>
+      <c r="N12" t="str">
         <v>Y</v>
       </c>
     </row>
@@ -882,37 +940,43 @@
         <v>12</v>
       </c>
       <c r="B13" t="str">
-        <v>풍납시장</v>
+        <v>슬롯 #13 (12)추가</v>
       </c>
       <c r="C13" t="str">
+        <v>https://kstat.surveys.kr/2026/P26042401B/index.asp?KID=7SyhrpGqg&amp;type=tapi&amp;prid=2026070802&amp;mnid=900001346&amp;srt=1</v>
+      </c>
+      <c r="D13" t="str">
+        <v>풍납시장</v>
+      </c>
+      <c r="E13" t="str">
         <v>아트이븐프라자</v>
       </c>
-      <c r="D13" t="str">
+      <c r="F13" t="str">
         <v>219-01-88679</v>
       </c>
-      <c r="E13" t="str">
+      <c r="G13" t="str">
         <v>남궁민</v>
       </c>
-      <c r="F13" t="str">
+      <c r="H13" t="str">
         <v>02-484-8652</v>
       </c>
-      <c r="G13" t="str">
+      <c r="I13" t="str">
         <v>2022-02-03</v>
       </c>
-      <c r="H13" t="str">
+      <c r="J13" t="str">
         <v>가정용품 (종합 소매업 외 1개)</v>
       </c>
-      <c r="I13" t="str" xml:space="preserve">
-        <v xml:space="preserve">서울특별시 송파구
-주소정보 갱신</v>
-      </c>
-      <c r="J13" t="str">
-        <v>정상가맹</v>
-      </c>
-      <c r="K13" t="str">
-        <v>Y</v>
+      <c r="K13" t="str" xml:space="preserve">
+        <v xml:space="preserve">서울특별시 송파구
+주소정보 갱신</v>
       </c>
       <c r="L13" t="str">
+        <v>정상가맹</v>
+      </c>
+      <c r="M13" t="str">
+        <v>Y</v>
+      </c>
+      <c r="N13" t="str">
         <v>Y</v>
       </c>
     </row>
@@ -921,37 +985,43 @@
         <v>13</v>
       </c>
       <c r="B14" t="str">
-        <v>풍납시장</v>
+        <v>슬롯 #14 (13)추가</v>
       </c>
       <c r="C14" t="str">
+        <v>https://kstat.surveys.kr/2026/P26042401B/index.asp?KID=ngTrpE4bJ&amp;type=tapi&amp;prid=2026070802&amp;mnid=900001346&amp;srt=1</v>
+      </c>
+      <c r="D14" t="str">
+        <v>풍납시장</v>
+      </c>
+      <c r="E14" t="str">
         <v>서울침구</v>
       </c>
-      <c r="D14" t="str">
+      <c r="F14" t="str">
         <v>215-21-38215</v>
       </c>
-      <c r="E14" t="str">
-        <v/>
-      </c>
-      <c r="F14" t="str">
+      <c r="G14" t="str">
+        <v>-</v>
+      </c>
+      <c r="H14" t="str">
         <v>02-486-8300</v>
       </c>
-      <c r="G14" t="str">
+      <c r="I14" t="str">
         <v>2011-05-12</v>
       </c>
-      <c r="H14" t="str">
+      <c r="J14" t="str">
         <v>가정용품 (남자용 겉옷 소매업)</v>
       </c>
-      <c r="I14" t="str" xml:space="preserve">
-        <v xml:space="preserve">서울특별시 송파구
-주소정보 갱신</v>
-      </c>
-      <c r="J14" t="str">
-        <v>정상가맹</v>
-      </c>
-      <c r="K14" t="str">
-        <v>Y</v>
+      <c r="K14" t="str" xml:space="preserve">
+        <v xml:space="preserve">서울특별시 송파구
+주소정보 갱신</v>
       </c>
       <c r="L14" t="str">
+        <v>정상가맹</v>
+      </c>
+      <c r="M14" t="str">
+        <v>Y</v>
+      </c>
+      <c r="N14" t="str">
         <v>Y</v>
       </c>
     </row>
@@ -960,37 +1030,43 @@
         <v>14</v>
       </c>
       <c r="B15" t="str">
-        <v>풍납시장</v>
+        <v>슬롯 #15 (14)추가</v>
       </c>
       <c r="C15" t="str">
+        <v>https://kstat.surveys.kr/2026/P26042401B/index.asp?KID=a6l94Y3gX&amp;type=tapi&amp;prid=2026070802&amp;mnid=900001346&amp;srt=1</v>
+      </c>
+      <c r="D15" t="str">
+        <v>풍납시장</v>
+      </c>
+      <c r="E15" t="str">
         <v>덕인철물</v>
       </c>
-      <c r="D15" t="str">
+      <c r="F15" t="str">
         <v>219-01-27221</v>
       </c>
-      <c r="E15" t="str">
-        <v/>
-      </c>
-      <c r="F15" t="str">
+      <c r="G15" t="str">
+        <v>-</v>
+      </c>
+      <c r="H15" t="str">
         <v>02-2097-9797</v>
       </c>
-      <c r="G15" t="str">
+      <c r="I15" t="str">
         <v>2019-03-04</v>
       </c>
-      <c r="H15" t="str">
+      <c r="J15" t="str">
         <v>가정용품 (철물 및 난방용구 소매업)</v>
       </c>
-      <c r="I15" t="str" xml:space="preserve">
-        <v xml:space="preserve">서울특별시 송파구
-주소정보 갱신</v>
-      </c>
-      <c r="J15" t="str">
-        <v>정상가맹</v>
-      </c>
-      <c r="K15" t="str">
-        <v>Y</v>
+      <c r="K15" t="str" xml:space="preserve">
+        <v xml:space="preserve">서울특별시 송파구
+주소정보 갱신</v>
       </c>
       <c r="L15" t="str">
+        <v>정상가맹</v>
+      </c>
+      <c r="M15" t="str">
+        <v>Y</v>
+      </c>
+      <c r="N15" t="str">
         <v>Y</v>
       </c>
     </row>
@@ -999,37 +1075,43 @@
         <v>15</v>
       </c>
       <c r="B16" t="str">
-        <v>풍납시장</v>
+        <v>슬롯 #16 (15)추가</v>
       </c>
       <c r="C16" t="str">
+        <v>https://kstat.surveys.kr/2026/P26042401B/index.asp?KID=jfXJSXy5E&amp;type=tapi&amp;prid=2026070802&amp;mnid=900001346&amp;srt=1</v>
+      </c>
+      <c r="D16" t="str">
+        <v>풍납시장</v>
+      </c>
+      <c r="E16" t="str">
         <v>독도쭈꾸미</v>
       </c>
-      <c r="D16" t="str">
+      <c r="F16" t="str">
         <v>215-21-99736</v>
       </c>
-      <c r="E16" t="str">
-        <v/>
-      </c>
-      <c r="F16" t="str">
+      <c r="G16" t="str">
+        <v>-</v>
+      </c>
+      <c r="H16" t="str">
         <v>02-475-6204</v>
       </c>
-      <c r="G16" t="str">
+      <c r="I16" t="str">
         <v>2014-04-07</v>
       </c>
-      <c r="H16" t="str">
+      <c r="J16" t="str">
         <v>음식점업 (한식 일반 음식점업 외 1개)</v>
       </c>
-      <c r="I16" t="str" xml:space="preserve">
-        <v xml:space="preserve">서울특별시 송파구
-주소정보 갱신</v>
-      </c>
-      <c r="J16" t="str">
-        <v>정상가맹</v>
-      </c>
-      <c r="K16" t="str">
-        <v>Y</v>
+      <c r="K16" t="str" xml:space="preserve">
+        <v xml:space="preserve">서울특별시 송파구
+주소정보 갱신</v>
       </c>
       <c r="L16" t="str">
+        <v>정상가맹</v>
+      </c>
+      <c r="M16" t="str">
+        <v>Y</v>
+      </c>
+      <c r="N16" t="str">
         <v>Y</v>
       </c>
     </row>
@@ -1038,36 +1120,42 @@
         <v>16</v>
       </c>
       <c r="B17" t="str">
-        <v>풍납시장</v>
+        <v>슬롯 #17 (16)추가</v>
       </c>
       <c r="C17" t="str">
+        <v>https://kstat.surveys.kr/2026/P26042401B/index.asp?KID=NdlR9tVqG&amp;type=tapi&amp;prid=2026070802&amp;mnid=900001346&amp;srt=1</v>
+      </c>
+      <c r="D17" t="str">
+        <v>풍납시장</v>
+      </c>
+      <c r="E17" t="str">
         <v>어묵집</v>
       </c>
-      <c r="D17" t="str">
+      <c r="F17" t="str">
         <v>371-09-03237</v>
       </c>
-      <c r="E17" t="str">
-        <v/>
-      </c>
-      <c r="F17" t="str">
+      <c r="G17" t="str">
+        <v>-</v>
+      </c>
+      <c r="H17" t="str">
         <v>0507-1353-3610</v>
       </c>
-      <c r="G17" t="str">
+      <c r="I17" t="str">
         <v>2026-05-04</v>
       </c>
-      <c r="H17" t="str">
+      <c r="J17" t="str">
         <v>음식점업 (한식/일반음식점/분식)</v>
       </c>
-      <c r="I17" t="str">
+      <c r="K17" t="str">
         <v>서울특별시 송파구</v>
       </c>
-      <c r="J17" t="str">
-        <v>정상가맹</v>
-      </c>
-      <c r="K17" t="str">
-        <v>Y</v>
-      </c>
       <c r="L17" t="str">
+        <v>정상가맹</v>
+      </c>
+      <c r="M17" t="str">
+        <v>Y</v>
+      </c>
+      <c r="N17" t="str">
         <v>Y</v>
       </c>
     </row>
@@ -1076,37 +1164,43 @@
         <v>17</v>
       </c>
       <c r="B18" t="str">
-        <v>풍납시장</v>
+        <v>슬롯 #18 (17)추가</v>
       </c>
       <c r="C18" t="str">
+        <v>https://kstat.surveys.kr/2026/P26042401B/index.asp?KID=JqrhZwErQ&amp;type=tapi&amp;prid=2026070802&amp;mnid=900001346&amp;srt=1</v>
+      </c>
+      <c r="D18" t="str">
+        <v>풍납시장</v>
+      </c>
+      <c r="E18" t="str">
         <v>카페 3권역</v>
       </c>
-      <c r="D18" t="str">
+      <c r="F18" t="str">
         <v>422-31-01862</v>
       </c>
-      <c r="E18" t="str">
-        <v/>
-      </c>
-      <c r="F18" t="str">
+      <c r="G18" t="str">
+        <v>-</v>
+      </c>
+      <c r="H18" t="str">
         <v>0507-1474-0958</v>
       </c>
-      <c r="G18" t="str">
+      <c r="I18" t="str">
         <v>2026-05-21</v>
       </c>
-      <c r="H18" t="str">
+      <c r="J18" t="str">
         <v>음식점업 (한식/일반음식점/분식)</v>
       </c>
-      <c r="I18" t="str" xml:space="preserve">
-        <v xml:space="preserve">서울특별시 송파구
-주소정보 갱신</v>
-      </c>
-      <c r="J18" t="str">
-        <v>정상가맹</v>
-      </c>
-      <c r="K18" t="str">
-        <v>Y</v>
+      <c r="K18" t="str" xml:space="preserve">
+        <v xml:space="preserve">서울특별시 송파구
+주소정보 갱신</v>
       </c>
       <c r="L18" t="str">
+        <v>정상가맹</v>
+      </c>
+      <c r="M18" t="str">
+        <v>Y</v>
+      </c>
+      <c r="N18" t="str">
         <v>Y</v>
       </c>
     </row>
@@ -1115,37 +1209,43 @@
         <v>18</v>
       </c>
       <c r="B19" t="str">
-        <v>풍납시장</v>
+        <v>슬롯 #19 (18)추가</v>
       </c>
       <c r="C19" t="str">
+        <v>https://kstat.surveys.kr/2026/P26042401B/index.asp?KID=NjZZUh3EQ&amp;type=tapi&amp;prid=2026070802&amp;mnid=900001346&amp;srt=1</v>
+      </c>
+      <c r="D19" t="str">
+        <v>풍납시장</v>
+      </c>
+      <c r="E19" t="str">
         <v>메가엠지씨커피송파풍납시장점</v>
       </c>
-      <c r="D19" t="str">
+      <c r="F19" t="str">
         <v>701-10-02963</v>
       </c>
-      <c r="E19" t="str">
+      <c r="G19" t="str">
         <v>변희만</v>
       </c>
-      <c r="F19" t="str">
-        <v/>
-      </c>
-      <c r="G19" t="str">
+      <c r="H19" t="str">
+        <v>-</v>
+      </c>
+      <c r="I19" t="str">
         <v>2026-03-10</v>
       </c>
-      <c r="H19" t="str">
+      <c r="J19" t="str">
         <v>음식점업 (기타 비알코올 음료점업)</v>
       </c>
-      <c r="I19" t="str" xml:space="preserve">
-        <v xml:space="preserve">서울특별시 송파구
-주소정보 갱신</v>
-      </c>
-      <c r="J19" t="str">
-        <v>정상가맹</v>
-      </c>
-      <c r="K19" t="str">
-        <v>Y</v>
+      <c r="K19" t="str" xml:space="preserve">
+        <v xml:space="preserve">서울특별시 송파구
+주소정보 갱신</v>
       </c>
       <c r="L19" t="str">
+        <v>정상가맹</v>
+      </c>
+      <c r="M19" t="str">
+        <v>Y</v>
+      </c>
+      <c r="N19" t="str">
         <v>Y</v>
       </c>
     </row>
@@ -1154,37 +1254,43 @@
         <v>19</v>
       </c>
       <c r="B20" t="str">
-        <v>풍납시장</v>
+        <v>슬롯 #20 (19)추가</v>
       </c>
       <c r="C20" t="str">
+        <v>https://kstat.surveys.kr/2026/P26042401B/index.asp?KID=oJJjNC5No&amp;type=tapi&amp;prid=2026070802&amp;mnid=900001346&amp;srt=1</v>
+      </c>
+      <c r="D20" t="str">
+        <v>풍납시장</v>
+      </c>
+      <c r="E20" t="str">
         <v>예작</v>
       </c>
-      <c r="D20" t="str">
+      <c r="F20" t="str">
         <v>212-15-71233</v>
       </c>
-      <c r="E20" t="str">
-        <v/>
-      </c>
-      <c r="F20" t="str">
+      <c r="G20" t="str">
+        <v>-</v>
+      </c>
+      <c r="H20" t="str">
         <v>02-2147-2000</v>
       </c>
-      <c r="G20" t="str">
+      <c r="I20" t="str">
         <v>2012-07-12</v>
       </c>
-      <c r="H20" t="str">
+      <c r="J20" t="str">
         <v>기타소매 (두발 미용업)</v>
       </c>
-      <c r="I20" t="str" xml:space="preserve">
-        <v xml:space="preserve">서울특별시 송파구
-주소정보 갱신</v>
-      </c>
-      <c r="J20" t="str">
-        <v>정상가맹</v>
-      </c>
-      <c r="K20" t="str">
-        <v>Y</v>
+      <c r="K20" t="str" xml:space="preserve">
+        <v xml:space="preserve">서울특별시 송파구
+주소정보 갱신</v>
       </c>
       <c r="L20" t="str">
+        <v>정상가맹</v>
+      </c>
+      <c r="M20" t="str">
+        <v>Y</v>
+      </c>
+      <c r="N20" t="str">
         <v>Y</v>
       </c>
     </row>
@@ -1193,37 +1299,43 @@
         <v>20</v>
       </c>
       <c r="B21" t="str">
-        <v>풍납시장</v>
+        <v>슬롯 #21 (20)추가</v>
       </c>
       <c r="C21" t="str">
+        <v>https://kstat.surveys.kr/2026/P26042401B/index.asp?KID=4cwi7xkAU&amp;type=tapi&amp;prid=2026070802&amp;mnid=900001346&amp;srt=1</v>
+      </c>
+      <c r="D21" t="str">
+        <v>풍납시장</v>
+      </c>
+      <c r="E21" t="str">
         <v>건강지킴이</v>
       </c>
-      <c r="D21" t="str">
+      <c r="F21" t="str">
         <v>495-07-02656</v>
       </c>
-      <c r="E21" t="str">
+      <c r="G21" t="str">
         <v>박현주</v>
       </c>
-      <c r="F21" t="str">
+      <c r="H21" t="str">
         <v>02-2133-6105</v>
       </c>
-      <c r="G21" t="str">
+      <c r="I21" t="str">
         <v>2024-07-19</v>
       </c>
-      <c r="H21" t="str">
+      <c r="J21" t="str">
         <v>기타소매 (피부 미용업)</v>
       </c>
-      <c r="I21" t="str" xml:space="preserve">
-        <v xml:space="preserve">서울특별시 송파구
-주소정보 갱신</v>
-      </c>
-      <c r="J21" t="str">
-        <v>정상가맹</v>
-      </c>
-      <c r="K21" t="str">
-        <v>Y</v>
+      <c r="K21" t="str" xml:space="preserve">
+        <v xml:space="preserve">서울특별시 송파구
+주소정보 갱신</v>
       </c>
       <c r="L21" t="str">
+        <v>정상가맹</v>
+      </c>
+      <c r="M21" t="str">
+        <v>Y</v>
+      </c>
+      <c r="N21" t="str">
         <v>N</v>
       </c>
     </row>
@@ -1232,36 +1344,42 @@
         <v>21</v>
       </c>
       <c r="B22" t="str">
-        <v>풍납시장</v>
+        <v>슬롯 #22 (21)추가</v>
       </c>
       <c r="C22" t="str">
+        <v>https://kstat.surveys.kr/2026/P26042401B/index.asp?KID=bOITDPyUG&amp;type=tapi&amp;prid=2026070802&amp;mnid=900001346&amp;srt=1</v>
+      </c>
+      <c r="D22" t="str">
+        <v>풍납시장</v>
+      </c>
+      <c r="E22" t="str">
         <v>큐사랑(풍납시장점)</v>
       </c>
-      <c r="D22" t="str">
+      <c r="F22" t="str">
         <v>460-39-01424</v>
       </c>
-      <c r="E22" t="str">
-        <v/>
-      </c>
-      <c r="F22" t="str">
+      <c r="G22" t="str">
+        <v>-</v>
+      </c>
+      <c r="H22" t="str">
         <v>0507-1484-0613</v>
       </c>
-      <c r="G22" t="str">
+      <c r="I22" t="str">
         <v>2026-08-05</v>
       </c>
-      <c r="H22" t="str">
+      <c r="J22" t="str">
         <v>기타소매 (안경/약국/생활소매업)</v>
       </c>
-      <c r="I22" t="str">
+      <c r="K22" t="str">
         <v>서울특별시 송파구</v>
       </c>
-      <c r="J22" t="str">
-        <v>정상가맹</v>
-      </c>
-      <c r="K22" t="str">
-        <v>Y</v>
-      </c>
       <c r="L22" t="str">
+        <v>정상가맹</v>
+      </c>
+      <c r="M22" t="str">
+        <v>Y</v>
+      </c>
+      <c r="N22" t="str">
         <v>Y</v>
       </c>
     </row>
@@ -1270,37 +1388,43 @@
         <v>22</v>
       </c>
       <c r="B23" t="str">
-        <v>풍납시장</v>
+        <v>슬롯 #23 (22)추가</v>
       </c>
       <c r="C23" t="str">
+        <v>https://kstat.surveys.kr/2026/P26042401B/index.asp?KID=FOOkcSy06&amp;type=tapi&amp;prid=2026070802&amp;mnid=900001346&amp;srt=1</v>
+      </c>
+      <c r="D23" t="str">
+        <v>풍납시장</v>
+      </c>
+      <c r="E23" t="str">
         <v>풍납배내과</v>
       </c>
-      <c r="D23" t="str">
+      <c r="F23" t="str">
         <v>215-91-72652</v>
       </c>
-      <c r="E23" t="str">
-        <v/>
-      </c>
-      <c r="F23" t="str">
+      <c r="G23" t="str">
+        <v>-</v>
+      </c>
+      <c r="H23" t="str">
         <v>02-470-4778</v>
       </c>
-      <c r="G23" t="str">
+      <c r="I23" t="str">
         <v>2026-04-08</v>
       </c>
-      <c r="H23" t="str">
+      <c r="J23" t="str">
         <v>근린상권 (병원 외 1개)</v>
       </c>
-      <c r="I23" t="str" xml:space="preserve">
-        <v xml:space="preserve">서울특별시 송파구
-주소정보 갱신</v>
-      </c>
-      <c r="J23" t="str">
-        <v>정상가맹</v>
-      </c>
-      <c r="K23" t="str">
-        <v>Y</v>
+      <c r="K23" t="str" xml:space="preserve">
+        <v xml:space="preserve">서울특별시 송파구
+주소정보 갱신</v>
       </c>
       <c r="L23" t="str">
+        <v>정상가맹</v>
+      </c>
+      <c r="M23" t="str">
+        <v>Y</v>
+      </c>
+      <c r="N23" t="str">
         <v>Y</v>
       </c>
     </row>
@@ -1309,37 +1433,43 @@
         <v>23</v>
       </c>
       <c r="B24" t="str">
-        <v>풍납시장</v>
+        <v>슬롯 #24 (23)추가</v>
       </c>
       <c r="C24" t="str">
+        <v>https://kstat.surveys.kr/2026/P26042401B/index.asp?KID=OH7Lypweo&amp;type=tapi&amp;prid=2026070802&amp;mnid=900001346&amp;srt=1</v>
+      </c>
+      <c r="D24" t="str">
+        <v>풍납시장</v>
+      </c>
+      <c r="E24" t="str">
         <v xml:space="preserve">리안헤어천호역점 </v>
       </c>
-      <c r="D24" t="str">
+      <c r="F24" t="str">
         <v>781-27-00294</v>
       </c>
-      <c r="E24" t="str">
-        <v/>
-      </c>
-      <c r="F24" t="str">
+      <c r="G24" t="str">
+        <v>-</v>
+      </c>
+      <c r="H24" t="str">
         <v>02-471-2333</v>
       </c>
-      <c r="G24" t="str">
+      <c r="I24" t="str">
         <v>2020-04-09</v>
       </c>
-      <c r="H24" t="str">
+      <c r="J24" t="str">
         <v>근린상권 (두발 미용업)</v>
       </c>
-      <c r="I24" t="str" xml:space="preserve">
-        <v xml:space="preserve">서울특별시 송파구
-주소정보 갱신</v>
-      </c>
-      <c r="J24" t="str">
-        <v>정상가맹</v>
-      </c>
-      <c r="K24" t="str">
-        <v>Y</v>
+      <c r="K24" t="str" xml:space="preserve">
+        <v xml:space="preserve">서울특별시 송파구
+주소정보 갱신</v>
       </c>
       <c r="L24" t="str">
+        <v>정상가맹</v>
+      </c>
+      <c r="M24" t="str">
+        <v>Y</v>
+      </c>
+      <c r="N24" t="str">
         <v>Y</v>
       </c>
     </row>
@@ -1348,43 +1478,49 @@
         <v>24</v>
       </c>
       <c r="B25" t="str">
-        <v>풍납시장</v>
+        <v>슬롯 #25 (24)추가</v>
       </c>
       <c r="C25" t="str">
+        <v>https://kstat.surveys.kr/2026/P26042401B/index.asp?KID=GycZZf28Z&amp;type=tapi&amp;prid=2026070802&amp;mnid=900001346&amp;srt=1</v>
+      </c>
+      <c r="D25" t="str">
+        <v>풍납시장</v>
+      </c>
+      <c r="E25" t="str">
         <v>바르다네일</v>
       </c>
-      <c r="D25" t="str">
+      <c r="F25" t="str">
         <v>808-05-00393</v>
       </c>
-      <c r="E25" t="str">
-        <v/>
-      </c>
-      <c r="F25" t="str">
+      <c r="G25" t="str">
+        <v>-</v>
+      </c>
+      <c r="H25" t="str">
         <v>02-471-9403</v>
       </c>
-      <c r="G25" t="str">
+      <c r="I25" t="str">
         <v>2025-07-24</v>
       </c>
-      <c r="H25" t="str">
+      <c r="J25" t="str">
         <v>근린상권 (기타 미용업)</v>
       </c>
-      <c r="I25" t="str" xml:space="preserve">
-        <v xml:space="preserve">서울특별시 송파구
-주소정보 갱신</v>
-      </c>
-      <c r="J25" t="str">
-        <v>정상가맹</v>
-      </c>
-      <c r="K25" t="str">
-        <v>Y</v>
+      <c r="K25" t="str" xml:space="preserve">
+        <v xml:space="preserve">서울특별시 송파구
+주소정보 갱신</v>
       </c>
       <c r="L25" t="str">
+        <v>정상가맹</v>
+      </c>
+      <c r="M25" t="str">
+        <v>Y</v>
+      </c>
+      <c r="N25" t="str">
         <v>Y</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:L25"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:N25"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>